<commit_message>
fix(booking): allow completion with skipped or partial optional sections (Row 44)
- Step 3 (Live Stalls):
  - Make Live Stall step optional in stepValid(3) so customers can advance without live stalls.
  - Update liveNext to allow continuing to Step 4 past the last live stall category.
  - Add explicit "Skip Live Stalls" actions in StepMenu banner and MenuStepNav.

- Step 4 (Add-ons & Extras) & Partial Courses:
  - Update orderHasItems so choosing a feast package and caterer enables completion even if optional Live Stalls and Add-ons are left unselected.
  - Preserve strict validation on required fields (Package selection, Occasion, Event Date meeting lead notice, Guest limits, and Contact info).

- Progress Tracker:
  - Mark Row 44 as Completed in Bhojpatra_Progress_Tracker.xlsx.
</commit_message>
<xml_diff>
--- a/Bhojpatra_Progress_Tracker.xlsx
+++ b/Bhojpatra_Progress_Tracker.xlsx
@@ -1340,10 +1340,10 @@
       </c>
       <c r="B44" s="5"/>
       <c r="C44" s="17" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="D44" s="17" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="E44" s="9"/>
     </row>

</xml_diff>